<commit_message>
Regenerate the pipeline-3 summary sheets against the current presets
test_checked_in_sheet_matches_its_summary_preset failed for all three
sheets since #1623 (pulse_time_begin on every history preset) and #1751
(beta_volume_B2, beta_normal_B2, normalized_plasma_current on
equilibrium_global). equilibrium_global_history.xlsx is rebuilt from the
main source (shots 39000-48500: 1377 shots, 8772 rows). The
volume_averaged and core_profiles presets read core_profiles, which the
main source no longer carries for any of these shots (#1842), so those two
sheets are rebuilt from the legacy public source exactly as the 2026-08-26
sheets were (6 and 3 shots).

Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/workflow/automatic_pipeline_3_data_summary/volume_averaged_parameters.xlsx
+++ b/workflow/automatic_pipeline_3_data_summary/volume_averaged_parameters.xlsx
@@ -2,15 +2,14 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
-  <workbookProtection/>
   <bookViews>
-    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
+    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="240" yWindow="15" windowWidth="16095" windowHeight="9660" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Sheet1'!$A$1:$K$13</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Sheet1'!$A$1:$L$16</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -18,7 +17,9 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="0"/>
+  <numFmts count="1">
+    <numFmt numFmtId="164" formatCode="0.000"/>
+  </numFmts>
   <fonts count="2">
     <font>
       <name val="Calibri"/>
@@ -57,12 +58,14 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="1" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
-    <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
+    <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
   <colors>
@@ -425,20 +428,21 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K13"/>
+  <dimension ref="A1:L16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
-    <col width="12" customWidth="1" min="2" max="2"/>
+    <col width="18" customWidth="1" min="2" max="2"/>
     <col width="12" customWidth="1" min="3" max="3"/>
-    <col width="13" customWidth="1" min="4" max="4"/>
-    <col width="20" customWidth="1" min="5" max="5"/>
-    <col width="13" customWidth="1" min="6" max="6"/>
-    <col width="14" customWidth="1" min="7" max="7"/>
+    <col width="12" customWidth="1" min="4" max="4"/>
+    <col width="13" customWidth="1" min="5" max="5"/>
+    <col width="20" customWidth="1" min="6" max="6"/>
+    <col width="13" customWidth="1" min="7" max="7"/>
     <col width="14" customWidth="1" min="8" max="8"/>
-    <col width="24" customWidth="1" min="9" max="9"/>
+    <col width="14" customWidth="1" min="9" max="9"/>
     <col width="24" customWidth="1" min="10" max="10"/>
     <col width="24" customWidth="1" min="11" max="11"/>
+    <col width="24" customWidth="1" min="12" max="12"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -449,477 +453,587 @@
       </c>
       <c r="B1" s="1" t="inlineStr">
         <is>
+          <t>pulse_time_begin</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
           <t>cp_index</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="D1" s="1" t="inlineStr">
         <is>
           <t>eq_index</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>time_core_s</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="F1" s="1" t="inlineStr">
         <is>
           <t>time_equilibrium_s</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="G1" s="1" t="inlineStr">
         <is>
           <t>time_diff_s</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="H1" s="1" t="inlineStr">
         <is>
           <t>ne_volume_m3</t>
         </is>
       </c>
-      <c r="H1" s="1" t="inlineStr">
+      <c r="I1" s="1" t="inlineStr">
         <is>
           <t>te_volume_eV</t>
         </is>
       </c>
-      <c r="I1" s="1" t="inlineStr">
+      <c r="J1" s="1" t="inlineStr">
         <is>
           <t>electron_pressure_volume_Pa</t>
         </is>
       </c>
-      <c r="J1" s="1" t="inlineStr">
+      <c r="K1" s="1" t="inlineStr">
         <is>
           <t>equilibrium_pressure_volume_Pa</t>
         </is>
       </c>
-      <c r="K1" s="1" t="inlineStr">
+      <c r="L1" s="1" t="inlineStr">
         <is>
           <t>electron_to_equilibrium_pressure_ratio</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" t="n">
+      <c r="A2" s="2" t="n">
+        <v>39915</v>
+      </c>
+      <c r="C2" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="D2" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="E2" s="3" t="n">
+        <v>0.316</v>
+      </c>
+      <c r="F2" s="3" t="n">
+        <v>0.316</v>
+      </c>
+      <c r="G2" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="H2" s="3" t="n">
+        <v>2.770392005620234e+18</v>
+      </c>
+      <c r="I2" s="3" t="n">
+        <v>105.7440809326004</v>
+      </c>
+      <c r="J2" s="3" t="n">
+        <v>93.87234816530163</v>
+      </c>
+      <c r="K2" s="3" t="n">
+        <v>10.71904311372206</v>
+      </c>
+      <c r="L2" s="3" t="n">
+        <v>8.757530608784498</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="2" t="n">
+        <v>39915</v>
+      </c>
+      <c r="C3" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="D3" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="E3" s="3" t="n">
+        <v>0.317</v>
+      </c>
+      <c r="F3" s="3" t="n">
+        <v>0.317</v>
+      </c>
+      <c r="G3" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="H3" s="3" t="n">
+        <v>3.123892042000352e+18</v>
+      </c>
+      <c r="I3" s="3" t="n">
+        <v>91.30157745665831</v>
+      </c>
+      <c r="J3" s="3" t="n">
+        <v>91.39336908312514</v>
+      </c>
+      <c r="K3" s="3" t="n">
+        <v>10.36872833214882</v>
+      </c>
+      <c r="L3" s="3" t="n">
+        <v>8.814327674084675</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="2" t="n">
         <v>39916</v>
       </c>
-      <c r="B2" t="n">
-        <v>0</v>
-      </c>
-      <c r="C2" t="n">
-        <v>0</v>
-      </c>
-      <c r="D2" t="n">
+      <c r="C4" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="D4" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="E4" s="3" t="n">
         <v>0.316</v>
       </c>
-      <c r="E2" t="n">
+      <c r="F4" s="3" t="n">
         <v>0.316</v>
       </c>
-      <c r="F2" t="n">
-        <v>0</v>
-      </c>
-      <c r="G2" t="n">
-        <v>2.48256711283123e+18</v>
-      </c>
-      <c r="H2" t="n">
-        <v>108.9476004141162</v>
-      </c>
-      <c r="I2" t="n">
-        <v>86.66805626116314</v>
-      </c>
-      <c r="J2" t="n">
-        <v>10.6096765291418</v>
-      </c>
-      <c r="K2" t="n">
-        <v>8.168774610904519</v>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="n">
+      <c r="G4" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="H4" s="3" t="n">
+        <v>2.482699587978707e+18</v>
+      </c>
+      <c r="I4" s="3" t="n">
+        <v>108.9528615190958</v>
+      </c>
+      <c r="J4" s="3" t="n">
+        <v>86.6768664999273</v>
+      </c>
+      <c r="K4" s="3" t="n">
+        <v>10.61026027558449</v>
+      </c>
+      <c r="L4" s="3" t="n">
+        <v>8.169155538943881</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="2" t="n">
         <v>39916</v>
       </c>
-      <c r="B3" t="n">
+      <c r="C5" s="2" t="n">
         <v>1</v>
       </c>
-      <c r="C3" t="n">
+      <c r="D5" s="2" t="n">
         <v>1</v>
       </c>
-      <c r="D3" t="n">
+      <c r="E5" s="3" t="n">
         <v>0.317</v>
       </c>
-      <c r="E3" t="n">
+      <c r="F5" s="3" t="n">
         <v>0.317</v>
       </c>
-      <c r="F3" t="n">
-        <v>0</v>
-      </c>
-      <c r="G3" t="n">
-        <v>3.29831274755034e+18</v>
-      </c>
-      <c r="H3" t="n">
-        <v>105.9473687431206</v>
-      </c>
-      <c r="I3" t="n">
-        <v>111.9753420930632</v>
-      </c>
-      <c r="J3" t="n">
-        <v>10.75214014011829</v>
-      </c>
-      <c r="K3" t="n">
-        <v>10.41423759677962</v>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="n">
+      <c r="G5" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="H5" s="3" t="n">
+        <v>3.298516714144583e+18</v>
+      </c>
+      <c r="I5" s="3" t="n">
+        <v>105.9533525540894</v>
+      </c>
+      <c r="J5" s="3" t="n">
+        <v>111.9885912685345</v>
+      </c>
+      <c r="K5" s="3" t="n">
+        <v>10.75281736114512</v>
+      </c>
+      <c r="L5" s="3" t="n">
+        <v>10.41481385829177</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="2" t="n">
         <v>39916</v>
       </c>
-      <c r="B4" t="n">
+      <c r="C6" s="2" t="n">
         <v>2</v>
       </c>
-      <c r="C4" t="n">
+      <c r="D6" s="2" t="n">
         <v>2</v>
       </c>
-      <c r="D4" t="n">
+      <c r="E6" s="3" t="n">
         <v>0.318</v>
       </c>
-      <c r="E4" t="n">
+      <c r="F6" s="3" t="n">
         <v>0.318</v>
       </c>
-      <c r="F4" t="n">
-        <v>0</v>
-      </c>
-      <c r="G4" t="n">
-        <v>3.175436480427231e+18</v>
-      </c>
-      <c r="H4" t="n">
-        <v>98.48554047856517</v>
-      </c>
-      <c r="I4" t="n">
-        <v>100.2112067127764</v>
-      </c>
-      <c r="J4" t="n">
-        <v>10.65795637401063</v>
-      </c>
-      <c r="K4" t="n">
-        <v>9.402478598724699</v>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="n">
+      <c r="G6" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="H6" s="3" t="n">
+        <v>3.175637437653519e+18</v>
+      </c>
+      <c r="I6" s="3" t="n">
+        <v>98.49138752124405</v>
+      </c>
+      <c r="J6" s="3" t="n">
+        <v>100.223498441657</v>
+      </c>
+      <c r="K6" s="3" t="n">
+        <v>10.65865931635853</v>
+      </c>
+      <c r="L6" s="3" t="n">
+        <v>9.403011717227661</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="2" t="n">
         <v>39916</v>
       </c>
-      <c r="B5" t="n">
+      <c r="C7" s="2" t="n">
         <v>3</v>
       </c>
-      <c r="C5" t="n">
+      <c r="D7" s="2" t="n">
         <v>3</v>
       </c>
-      <c r="D5" t="n">
+      <c r="E7" s="3" t="n">
         <v>0.319</v>
       </c>
-      <c r="E5" t="n">
+      <c r="F7" s="3" t="n">
         <v>0.319</v>
       </c>
-      <c r="F5" t="n">
-        <v>0</v>
-      </c>
-      <c r="G5" t="n">
-        <v>2.279674710290394e+18</v>
-      </c>
-      <c r="H5" t="n">
-        <v>91.24317344384565</v>
-      </c>
-      <c r="I5" t="n">
-        <v>66.65207164007708</v>
-      </c>
-      <c r="J5" t="n">
-        <v>9.751233912589436</v>
-      </c>
-      <c r="K5" t="n">
-        <v>6.835244876448426</v>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" t="n">
+      <c r="G7" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="H7" s="3" t="n">
+        <v>2.279634101701252e+18</v>
+      </c>
+      <c r="I7" s="3" t="n">
+        <v>91.24119944475849</v>
+      </c>
+      <c r="J7" s="3" t="n">
+        <v>66.64944238741387</v>
+      </c>
+      <c r="K7" s="3" t="n">
+        <v>9.751066124065803</v>
+      </c>
+      <c r="L7" s="3" t="n">
+        <v>6.835092854403056</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="2" t="n">
         <v>39916</v>
       </c>
-      <c r="B6" t="n">
+      <c r="C8" s="2" t="n">
         <v>4</v>
       </c>
-      <c r="C6" t="n">
+      <c r="D8" s="2" t="n">
         <v>4</v>
       </c>
-      <c r="D6" t="n">
+      <c r="E8" s="3" t="n">
         <v>0.32</v>
       </c>
-      <c r="E6" t="n">
+      <c r="F8" s="3" t="n">
         <v>0.32</v>
       </c>
-      <c r="F6" t="n">
-        <v>0</v>
-      </c>
-      <c r="G6" t="n">
-        <v>3.232448301818398e+18</v>
-      </c>
-      <c r="H6" t="n">
-        <v>149.0968846542004</v>
-      </c>
-      <c r="I6" t="n">
-        <v>154.4331557824489</v>
-      </c>
-      <c r="J6" t="n">
-        <v>9.25332750325793</v>
-      </c>
-      <c r="K6" t="n">
-        <v>16.68947259546101</v>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" t="n">
+      <c r="G8" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="H8" s="3" t="n">
+        <v>3.232492246319317e+18</v>
+      </c>
+      <c r="I8" s="3" t="n">
+        <v>149.0983345725419</v>
+      </c>
+      <c r="J8" s="3" t="n">
+        <v>154.4367571031703</v>
+      </c>
+      <c r="K8" s="3" t="n">
+        <v>9.253467266381469</v>
+      </c>
+      <c r="L8" s="3" t="n">
+        <v>16.68960970600182</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="2" t="n">
         <v>39916</v>
       </c>
-      <c r="B7" t="n">
+      <c r="C9" s="2" t="n">
         <v>5</v>
       </c>
-      <c r="C7" t="n">
+      <c r="D9" s="2" t="n">
         <v>5</v>
       </c>
-      <c r="D7" t="n">
+      <c r="E9" s="3" t="n">
         <v>0.322</v>
       </c>
-      <c r="E7" t="n">
+      <c r="F9" s="3" t="n">
         <v>0.322</v>
       </c>
-      <c r="F7" t="n">
-        <v>0</v>
-      </c>
-      <c r="G7" t="n">
-        <v>5.970400908441853e+18</v>
-      </c>
-      <c r="H7" t="n">
-        <v>107.2652686553796</v>
-      </c>
-      <c r="I7" t="n">
-        <v>205.2121209099313</v>
-      </c>
-      <c r="J7" t="n">
-        <v>7.14785361466798</v>
-      </c>
-      <c r="K7" t="n">
-        <v>28.70961437833858</v>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" t="n">
+      <c r="G9" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="H9" s="3" t="n">
+        <v>5.970951570111389e+18</v>
+      </c>
+      <c r="I9" s="3" t="n">
+        <v>107.2758120849931</v>
+      </c>
+      <c r="J9" s="3" t="n">
+        <v>205.2512208064692</v>
+      </c>
+      <c r="K9" s="3" t="n">
+        <v>7.148585156117797</v>
+      </c>
+      <c r="L9" s="3" t="n">
+        <v>28.71214601546911</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="2" t="n">
         <v>39916</v>
       </c>
-      <c r="B8" t="n">
+      <c r="C10" s="2" t="n">
         <v>6</v>
       </c>
-      <c r="C8" t="n">
+      <c r="D10" s="2" t="n">
         <v>6</v>
       </c>
-      <c r="D8" t="n">
+      <c r="E10" s="3" t="n">
         <v>0.325</v>
       </c>
-      <c r="E8" t="n">
+      <c r="F10" s="3" t="n">
         <v>0.325</v>
       </c>
-      <c r="F8" t="n">
-        <v>0</v>
-      </c>
-      <c r="G8" t="n">
-        <v>6.074450785074559e+18</v>
-      </c>
-      <c r="H8" t="n">
-        <v>245.7242144199252</v>
-      </c>
-      <c r="I8" t="n">
-        <v>478.2944731435486</v>
-      </c>
-      <c r="J8" t="n">
-        <v>4.077501108036254</v>
-      </c>
-      <c r="K8" t="n">
-        <v>117.3008812188644</v>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" t="n">
+      <c r="G10" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="H10" s="3" t="n">
+        <v>6.074394177922189e+18</v>
+      </c>
+      <c r="I10" s="3" t="n">
+        <v>245.7226241417038</v>
+      </c>
+      <c r="J10" s="3" t="n">
+        <v>478.2869205710746</v>
+      </c>
+      <c r="K10" s="3" t="n">
+        <v>4.077498210029662</v>
+      </c>
+      <c r="L10" s="3" t="n">
+        <v>117.2991123318225</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="2" t="n">
         <v>39917</v>
       </c>
-      <c r="B9" t="n">
-        <v>0</v>
-      </c>
-      <c r="C9" t="n">
+      <c r="C11" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="D11" s="2" t="n">
         <v>6</v>
       </c>
-      <c r="D9" t="n">
+      <c r="E11" s="3" t="n">
         <v>0.325</v>
       </c>
-      <c r="E9" t="n">
+      <c r="F11" s="3" t="n">
         <v>0.325</v>
       </c>
-      <c r="F9" t="n">
-        <v>0</v>
-      </c>
-      <c r="G9" t="n">
-        <v>1.055727976900242e+19</v>
-      </c>
-      <c r="H9" t="n">
-        <v>300.0828397855231</v>
-      </c>
-      <c r="I9" t="n">
-        <v>1015.157858683784</v>
-      </c>
-      <c r="J9" t="n">
-        <v>2.264002289516206</v>
-      </c>
-      <c r="K9" t="n">
-        <v>448.3908268929854</v>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" t="n">
+      <c r="G11" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="H11" s="3" t="n">
+        <v>1.055810580293241e+19</v>
+      </c>
+      <c r="I11" s="3" t="n">
+        <v>300.1068330317447</v>
+      </c>
+      <c r="J11" s="3" t="n">
+        <v>1015.31846145906</v>
+      </c>
+      <c r="K11" s="3" t="n">
+        <v>2.264196425846463</v>
+      </c>
+      <c r="L11" s="3" t="n">
+        <v>448.4233125133949</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="2" t="n">
+        <v>40329</v>
+      </c>
+      <c r="C12" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="D12" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="E12" s="3" t="n">
+        <v>0.322</v>
+      </c>
+      <c r="F12" s="3" t="n">
+        <v>0.322</v>
+      </c>
+      <c r="G12" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="H12" s="3" t="n">
+        <v>1.631124558321377e+19</v>
+      </c>
+      <c r="I12" s="3" t="n">
+        <v>38.46440964980435</v>
+      </c>
+      <c r="J12" s="3" t="n">
+        <v>201.0419033366544</v>
+      </c>
+      <c r="K12" s="3" t="n">
+        <v>4.179104461082509</v>
+      </c>
+      <c r="L12" s="3" t="n">
+        <v>48.10645563154427</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="2" t="n">
         <v>40330</v>
       </c>
-      <c r="B10" t="n">
-        <v>0</v>
-      </c>
-      <c r="C10" t="n">
-        <v>0</v>
-      </c>
-      <c r="D10" t="n">
+      <c r="C13" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="D13" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="E13" s="3" t="n">
         <v>0.32</v>
       </c>
-      <c r="E10" t="n">
+      <c r="F13" s="3" t="n">
         <v>0.32</v>
       </c>
-      <c r="F10" t="n">
-        <v>0</v>
-      </c>
-      <c r="G10" t="n">
-        <v>1.272278252560573e+19</v>
-      </c>
-      <c r="H10" t="n">
-        <v>32.27148906381752</v>
-      </c>
-      <c r="I10" t="n">
-        <v>131.565341726876</v>
-      </c>
-      <c r="J10" t="n">
-        <v>9.361924296040813</v>
-      </c>
-      <c r="K10" t="n">
-        <v>14.05323708743462</v>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" t="n">
+      <c r="G13" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="H13" s="3" t="n">
+        <v>1.272407731542776e+19</v>
+      </c>
+      <c r="I13" s="3" t="n">
+        <v>32.27472771066834</v>
+      </c>
+      <c r="J13" s="3" t="n">
+        <v>131.5919358045322</v>
+      </c>
+      <c r="K13" s="3" t="n">
+        <v>9.362915899639431</v>
+      </c>
+      <c r="L13" s="3" t="n">
+        <v>14.05458910611381</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="2" t="n">
         <v>40330</v>
       </c>
-      <c r="B11" t="n">
+      <c r="C14" s="2" t="n">
         <v>1</v>
       </c>
-      <c r="C11" t="n">
+      <c r="D14" s="2" t="n">
         <v>1</v>
       </c>
-      <c r="D11" t="n">
+      <c r="E14" s="3" t="n">
         <v>0.321</v>
       </c>
-      <c r="E11" t="n">
+      <c r="F14" s="3" t="n">
         <v>0.321</v>
       </c>
-      <c r="F11" t="n">
-        <v>0</v>
-      </c>
-      <c r="G11" t="n">
-        <v>1.428657492452764e+19</v>
-      </c>
-      <c r="H11" t="n">
-        <v>33.51875430741877</v>
-      </c>
-      <c r="I11" t="n">
-        <v>153.4462864915866</v>
-      </c>
-      <c r="J11" t="n">
-        <v>6.511557341578033</v>
-      </c>
-      <c r="K11" t="n">
-        <v>23.56522079776386</v>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" t="n">
+      <c r="G14" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="H14" s="3" t="n">
+        <v>1.428777154123582e+19</v>
+      </c>
+      <c r="I14" s="3" t="n">
+        <v>33.52151988047854</v>
+      </c>
+      <c r="J14" s="3" t="n">
+        <v>153.4718005064026</v>
+      </c>
+      <c r="K14" s="3" t="n">
+        <v>6.512127697100746</v>
+      </c>
+      <c r="L14" s="3" t="n">
+        <v>23.56707479411522</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="2" t="n">
         <v>40330</v>
       </c>
-      <c r="B12" t="n">
+      <c r="C15" s="2" t="n">
         <v>2</v>
       </c>
-      <c r="C12" t="n">
+      <c r="D15" s="2" t="n">
         <v>2</v>
       </c>
-      <c r="D12" t="n">
+      <c r="E15" s="3" t="n">
         <v>0.323</v>
       </c>
-      <c r="E12" t="n">
+      <c r="F15" s="3" t="n">
         <v>0.323</v>
       </c>
-      <c r="F12" t="n">
-        <v>0</v>
-      </c>
-      <c r="G12" t="n">
-        <v>3.290910299980738e+19</v>
-      </c>
-      <c r="H12" t="n">
-        <v>44.73322987738777</v>
-      </c>
-      <c r="I12" t="n">
-        <v>471.722608102176</v>
-      </c>
-      <c r="J12" t="n">
-        <v>2.884652836998861</v>
-      </c>
-      <c r="K12" t="n">
-        <v>163.528380972508</v>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" t="n">
+      <c r="G15" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="H15" s="3" t="n">
+        <v>3.291312308711154e+19</v>
+      </c>
+      <c r="I15" s="3" t="n">
+        <v>44.73887965897641</v>
+      </c>
+      <c r="J15" s="3" t="n">
+        <v>471.839818040344</v>
+      </c>
+      <c r="K15" s="3" t="n">
+        <v>2.88503020671734</v>
+      </c>
+      <c r="L15" s="3" t="n">
+        <v>163.5476179562138</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="2" t="n">
         <v>40331</v>
       </c>
-      <c r="B13" t="n">
-        <v>0</v>
-      </c>
-      <c r="C13" t="n">
-        <v>0</v>
-      </c>
-      <c r="D13" t="n">
+      <c r="C16" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="D16" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="E16" s="3" t="n">
         <v>0.322</v>
       </c>
-      <c r="E13" t="n">
+      <c r="F16" s="3" t="n">
         <v>0.322</v>
       </c>
-      <c r="F13" t="n">
-        <v>0</v>
-      </c>
-      <c r="G13" t="n">
-        <v>1.341148297852507e+19</v>
-      </c>
-      <c r="H13" t="n">
-        <v>27.48545490732402</v>
-      </c>
-      <c r="I13" t="n">
-        <v>118.1190978812897</v>
-      </c>
-      <c r="J13" t="n">
-        <v>3.973874379008013</v>
-      </c>
-      <c r="K13" t="n">
-        <v>29.72391339425667</v>
+      <c r="G16" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="H16" s="3" t="n">
+        <v>1.341184776228541e+19</v>
+      </c>
+      <c r="I16" s="3" t="n">
+        <v>27.48629463406834</v>
+      </c>
+      <c r="J16" s="3" t="n">
+        <v>118.1259194799123</v>
+      </c>
+      <c r="K16" s="3" t="n">
+        <v>3.974014119477785</v>
+      </c>
+      <c r="L16" s="3" t="n">
+        <v>29.72458474692961</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:K13"/>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <autoFilter ref="A1:L16"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>